<commit_message>
fixed moderator uploading more than given slot
</commit_message>
<xml_diff>
--- a/public/frontend/exportsamples/importparticipantsample.xlsx
+++ b/public/frontend/exportsamples/importparticipantsample.xlsx
@@ -24,37 +24,37 @@
     <t>Male</t>
   </si>
   <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>sdsd@fff.com</t>
+  </si>
+  <si>
+    <t>sdsd@fffff.com</t>
+  </si>
+  <si>
+    <t>David Oghi</t>
+  </si>
+  <si>
+    <t>Kehinde Sholadoye</t>
+  </si>
+  <si>
+    <t>a.asass@gmail.com</t>
+  </si>
+  <si>
     <t>Female</t>
   </si>
   <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Sex</t>
-  </si>
-  <si>
-    <t>sdsd@fff.com</t>
-  </si>
-  <si>
-    <t>sdsd@fffff.com</t>
-  </si>
-  <si>
-    <t>David Oghi</t>
-  </si>
-  <si>
-    <t>Kehinde Sholadoye</t>
-  </si>
-  <si>
-    <t>Tobi Sholaolape</t>
-  </si>
-  <si>
-    <t>s.ola@gmail.com</t>
+    <t>Sarah Akande Ajiboye</t>
   </si>
 </sst>
 </file>
@@ -412,24 +412,24 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>2367232</v>
@@ -440,10 +440,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>23267632</v>
@@ -454,16 +454,16 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>2323</v>
+      </c>
+      <c r="D4" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4">
-        <v>9999</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>